<commit_message>
feat: implement comprehensive traffic analysis pipeline with model pruning, benchmarking, and validation modules
</commit_message>
<xml_diff>
--- a/benchmark_results.xlsx
+++ b/benchmark_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="40">
   <si>
     <t>Model</t>
   </si>
@@ -52,43 +52,88 @@
     <t>Config</t>
   </si>
   <si>
+    <t>Pruning Type</t>
+  </si>
+  <si>
+    <t>Actual Sparsity</t>
+  </si>
+  <si>
+    <t>Timestamp</t>
+  </si>
+  <si>
+    <t>Torch Version</t>
+  </si>
+  <si>
+    <t>State Dict Match Info</t>
+  </si>
+  <si>
     <t>Compression Ratio</t>
   </si>
   <si>
     <t>Throughput (img/s)</t>
   </si>
   <si>
-    <t>Pruning Type</t>
+    <t>DETR</t>
   </si>
   <si>
     <t>YOLOV5S</t>
   </si>
   <si>
-    <t>YOLOV5</t>
-  </si>
-  <si>
-    <t>DETR</t>
-  </si>
-  <si>
     <t>Baseline FP32</t>
   </si>
   <si>
-    <t>Magnitude Pruned (30%)</t>
-  </si>
-  <si>
-    <t>Magnitude Pruned (50%)</t>
-  </si>
-  <si>
-    <t>Magnitude Pruned (70%)</t>
-  </si>
-  <si>
-    <t>INT8 Quantized</t>
-  </si>
-  <si>
-    <t>Magnitude</t>
-  </si>
-  <si>
-    <t>Quantization</t>
+    <t>Pruned magnitude (30%)</t>
+  </si>
+  <si>
+    <t>Pruned magnitude (50%)</t>
+  </si>
+  <si>
+    <t>Pruned magnitude (70%)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>magnitude</t>
+  </si>
+  <si>
+    <t>2026-06-24T21:29:10.065610</t>
+  </si>
+  <si>
+    <t>2026-06-24T21:29:30.727929</t>
+  </si>
+  <si>
+    <t>2026-06-24T21:29:51.750397</t>
+  </si>
+  <si>
+    <t>2026-06-24T21:30:36.229434</t>
+  </si>
+  <si>
+    <t>2026-06-24T21:27:40.563664</t>
+  </si>
+  <si>
+    <t>2026-06-24T21:28:19.422417</t>
+  </si>
+  <si>
+    <t>2026-06-24T21:28:32.160345</t>
+  </si>
+  <si>
+    <t>2026-06-24T21:28:46.593285</t>
+  </si>
+  <si>
+    <t>2.8.0+cu128</t>
+  </si>
+  <si>
+    <t>{'matched_keys_count': 458, 'missing_keys_count': 0, 'unexpected_keys_count': 0}</t>
+  </si>
+  <si>
+    <t>{'matched_keys_count': 558, 'missing_keys_count': 0, 'unexpected_keys_count': 262}</t>
+  </si>
+  <si>
+    <t>{'matched_keys_count': 349, 'missing_keys_count': 0, 'unexpected_keys_count': 0}</t>
+  </si>
+  <si>
+    <t>{'matched_keys_count': 409, 'missing_keys_count': 0, 'unexpected_keys_count': 284}</t>
   </si>
 </sst>
 </file>
@@ -446,10 +491,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -495,284 +540,489 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B2">
-        <v>7225885</v>
+        <v>41299541</v>
       </c>
       <c r="C2">
-        <v>16436019200</v>
+        <v>114245529600</v>
       </c>
       <c r="D2">
-        <v>27.56681442260743</v>
+        <v>158.7989082336426</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>5.105471997521818</v>
+        <v>24.42111999960616</v>
       </c>
       <c r="G2">
-        <v>195.8682763288874</v>
+        <v>40.94816290227995</v>
       </c>
       <c r="H2">
+        <v>0.05192786069651741</v>
+      </c>
+      <c r="I2">
+        <v>0.04685746352413019</v>
+      </c>
+      <c r="J2">
+        <v>0.001995411903763041</v>
+      </c>
+      <c r="K2">
+        <v>0.0006302592650451538</v>
+      </c>
+      <c r="L2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N2">
         <v>0</v>
       </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2" t="s">
-        <v>18</v>
-      </c>
-      <c r="M2">
+      <c r="O2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>36</v>
+      </c>
+      <c r="R2">
         <v>1</v>
       </c>
-      <c r="N2">
-        <v>195.8682763288874</v>
+      <c r="S2">
+        <v>40.94816290227995</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B3">
-        <v>7225885</v>
+        <v>41299541</v>
       </c>
       <c r="C3">
-        <v>16436019200</v>
+        <v>114245529600</v>
       </c>
       <c r="D3">
-        <v>55.09002304077149</v>
+        <v>158.7989082336426</v>
       </c>
       <c r="E3">
         <v>0.3</v>
       </c>
       <c r="F3">
-        <v>4.610764000099152</v>
+        <v>23.41993000009097</v>
       </c>
       <c r="G3">
-        <v>216.8837962599031</v>
+        <v>42.6986758711967</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>0.05234933605720123</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>0.05751964085297419</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>0.001477842532421738</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>0.0005510098814222742</v>
       </c>
       <c r="L3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N3">
+        <v>0.3000000105555959</v>
+      </c>
+      <c r="O3" t="s">
+        <v>28</v>
+      </c>
+      <c r="P3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>37</v>
+      </c>
+      <c r="R3">
+        <v>1.428571428571429</v>
+      </c>
+      <c r="S3">
+        <v>42.6986758711967</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19">
+      <c r="A4" t="s">
         <v>19</v>
       </c>
-      <c r="M3">
-        <v>0.5003561605950178</v>
-      </c>
-      <c r="N3">
-        <v>216.8837962599031</v>
-      </c>
-      <c r="O3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
       <c r="B4">
-        <v>7225885</v>
+        <v>41299541</v>
       </c>
       <c r="C4">
-        <v>16436019200</v>
+        <v>114245529600</v>
       </c>
       <c r="D4">
-        <v>55.09002304077149</v>
+        <v>158.7989082336426</v>
       </c>
       <c r="E4">
         <v>0.5</v>
       </c>
       <c r="F4">
-        <v>4.837188003584743</v>
+        <v>28.60731399967335</v>
       </c>
       <c r="G4">
-        <v>206.7316794920768</v>
+        <v>34.95609549402011</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>0.03708243947287772</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>0.06790123456790123</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>0.0002706140462289725</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>0.0001039895973293782</v>
       </c>
       <c r="L4" t="s">
-        <v>20</v>
-      </c>
-      <c r="M4">
-        <v>0.5003561605950178</v>
+        <v>23</v>
+      </c>
+      <c r="M4" t="s">
+        <v>26</v>
       </c>
       <c r="N4">
-        <v>206.7316794920768</v>
+        <v>0.5</v>
       </c>
       <c r="O4" t="s">
-        <v>23</v>
+        <v>29</v>
+      </c>
+      <c r="P4" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>37</v>
+      </c>
+      <c r="R4">
+        <v>2</v>
+      </c>
+      <c r="S4">
+        <v>34.95609549402011</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B5">
-        <v>7225885</v>
+        <v>41299541</v>
       </c>
       <c r="C5">
-        <v>16436019200</v>
+        <v>114245529600</v>
       </c>
       <c r="D5">
-        <v>55.09002304077149</v>
+        <v>158.7989082336426</v>
       </c>
       <c r="E5">
         <v>0.7</v>
       </c>
       <c r="F5">
-        <v>4.556549997068942</v>
+        <v>23.10625799873378</v>
       </c>
       <c r="G5">
-        <v>219.4642878149615</v>
+        <v>43.27831880241274</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>0.009339080459770116</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>0.01094276094276094</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>7.993137355443698E-06</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>3.670846600588143E-06</v>
       </c>
       <c r="L5" t="s">
-        <v>21</v>
-      </c>
-      <c r="M5">
-        <v>0.5003561605950178</v>
+        <v>24</v>
+      </c>
+      <c r="M5" t="s">
+        <v>26</v>
       </c>
       <c r="N5">
-        <v>219.4642878149615</v>
+        <v>0.6999999894444041</v>
       </c>
       <c r="O5" t="s">
-        <v>23</v>
+        <v>30</v>
+      </c>
+      <c r="P5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>37</v>
+      </c>
+      <c r="R5">
+        <v>3.333333333333333</v>
+      </c>
+      <c r="S5">
+        <v>43.27831880241274</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:19">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B6">
-        <v>338530</v>
+        <v>7235389</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>16625254400</v>
       </c>
       <c r="D6">
-        <v>0.4</v>
+        <v>27.67383193969727</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
       <c r="F6">
-        <v>26.1</v>
+        <v>6.685178002808243</v>
       </c>
       <c r="G6">
-        <v>38.2</v>
+        <v>149.5846482442098</v>
       </c>
       <c r="H6">
-        <v>0.823</v>
+        <v>0.4313151637095299</v>
       </c>
       <c r="I6">
-        <v>0.8</v>
+        <v>0.6616161616161617</v>
       </c>
       <c r="J6">
-        <v>0.823</v>
+        <v>0.5136537030571721</v>
       </c>
       <c r="K6">
-        <v>0.5</v>
+        <v>0.3578119810724223</v>
       </c>
       <c r="L6" t="s">
-        <v>22</v>
-      </c>
-      <c r="M6">
-        <v>3.38</v>
+        <v>21</v>
+      </c>
+      <c r="M6" t="s">
+        <v>25</v>
       </c>
       <c r="N6">
-        <v>38.2</v>
+        <v>3.1875310437806E-06</v>
       </c>
       <c r="O6" t="s">
-        <v>24</v>
+        <v>31</v>
+      </c>
+      <c r="P6" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>38</v>
+      </c>
+      <c r="R6">
+        <v>1</v>
+      </c>
+      <c r="S6">
+        <v>149.5846482442098</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:19">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B7">
-        <v>71984</v>
+        <v>7235389</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>16625254400</v>
       </c>
       <c r="D7">
-        <v>0.11</v>
+        <v>27.67383193969727</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="F7">
-        <v>393.9</v>
+        <v>6.784187997691333</v>
       </c>
       <c r="G7">
-        <v>2.37</v>
+        <v>147.4015755961216</v>
       </c>
       <c r="H7">
-        <v>0.77</v>
+        <v>0.4198994252873563</v>
       </c>
       <c r="I7">
-        <v>0.76</v>
+        <v>0.6560044893378226</v>
       </c>
       <c r="J7">
-        <v>0.77</v>
+        <v>0.5094602831924128</v>
       </c>
       <c r="K7">
-        <v>0.43</v>
+        <v>0.3462508636069907</v>
       </c>
       <c r="L7" t="s">
         <v>22</v>
       </c>
-      <c r="M7">
-        <v>2.72</v>
+      <c r="M7" t="s">
+        <v>26</v>
       </c>
       <c r="N7">
-        <v>2.37</v>
+        <v>0.3000000277176613</v>
       </c>
       <c r="O7" t="s">
+        <v>32</v>
+      </c>
+      <c r="P7" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>39</v>
+      </c>
+      <c r="R7">
+        <v>1.428571428571429</v>
+      </c>
+      <c r="S7">
+        <v>147.4015755961216</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8">
+        <v>7235389</v>
+      </c>
+      <c r="C8">
+        <v>16625254400</v>
+      </c>
+      <c r="D8">
+        <v>27.67383193969727</v>
+      </c>
+      <c r="E8">
+        <v>0.5</v>
+      </c>
+      <c r="F8">
+        <v>5.928600000333972</v>
+      </c>
+      <c r="G8">
+        <v>168.6738858994818</v>
+      </c>
+      <c r="H8">
+        <v>0.398490704951224</v>
+      </c>
+      <c r="I8">
+        <v>0.6074635241301908</v>
+      </c>
+      <c r="J8">
+        <v>0.451417532096466</v>
+      </c>
+      <c r="K8">
+        <v>0.2887226123134802</v>
+      </c>
+      <c r="L8" t="s">
+        <v>23</v>
+      </c>
+      <c r="M8" t="s">
+        <v>26</v>
+      </c>
+      <c r="N8">
+        <v>0.5</v>
+      </c>
+      <c r="O8" t="s">
+        <v>33</v>
+      </c>
+      <c r="P8" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>39</v>
+      </c>
+      <c r="R8">
+        <v>2</v>
+      </c>
+      <c r="S8">
+        <v>168.6738858994818</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9">
+        <v>7235389</v>
+      </c>
+      <c r="C9">
+        <v>16625254400</v>
+      </c>
+      <c r="D9">
+        <v>27.67383193969727</v>
+      </c>
+      <c r="E9">
+        <v>0.7</v>
+      </c>
+      <c r="F9">
+        <v>5.782500000204891</v>
+      </c>
+      <c r="G9">
+        <v>172.9355814897652</v>
+      </c>
+      <c r="H9">
+        <v>0.4647302904564315</v>
+      </c>
+      <c r="I9">
+        <v>0.1885521885521886</v>
+      </c>
+      <c r="J9">
+        <v>0.1077460404597087</v>
+      </c>
+      <c r="K9">
+        <v>0.0662890946750074</v>
+      </c>
+      <c r="L9" t="s">
         <v>24</v>
+      </c>
+      <c r="M9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N9">
+        <v>0.6999999722823388</v>
+      </c>
+      <c r="O9" t="s">
+        <v>34</v>
+      </c>
+      <c r="P9" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>39</v>
+      </c>
+      <c r="R9">
+        <v>3.333333333333333</v>
+      </c>
+      <c r="S9">
+        <v>172.9355814897652</v>
       </c>
     </row>
   </sheetData>

</xml_diff>